<commit_message>
fix viewing of adjustment
</commit_message>
<xml_diff>
--- a/uploads/excel/bulk_upload_sales_merge.xlsx
+++ b/uploads/excel/bulk_upload_sales_merge.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12015" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12015"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="12">
   <si>
     <t>Reference Number</t>
   </si>
@@ -39,18 +39,12 @@
     <t>Invoice Number</t>
   </si>
   <si>
-    <t>TS-WF-219F-0030024</t>
-  </si>
-  <si>
     <t>1590EC</t>
   </si>
   <si>
     <t>Reference No</t>
   </si>
   <si>
-    <t>TS-WF-234F-0050149</t>
-  </si>
-  <si>
     <t>sales_merge_transaction_head</t>
   </si>
   <si>
@@ -61,13 +55,19 @@
   </si>
   <si>
     <t>to update if checker exist</t>
+  </si>
+  <si>
+    <t>TS-WF-236F-0053107</t>
+  </si>
+  <si>
+    <t>TS-WF-236F-0053347</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -95,13 +95,6 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -123,13 +116,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -410,48 +402,55 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.5703125" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.5703125" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="4">
-        <v>1001</v>
+      <c r="C2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="4">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="4">
+        <v>789</v>
       </c>
     </row>
   </sheetData>
@@ -470,21 +469,21 @@
         <v>0</v>
       </c>
       <c r="F32" t="s">
+        <v>6</v>
+      </c>
+      <c r="G32" t="s">
         <v>8</v>
-      </c>
-      <c r="G32" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="33" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E33" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34" spans="5:7" x14ac:dyDescent="0.25">
@@ -492,10 +491,10 @@
         <v>1</v>
       </c>
       <c r="F34" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G34" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35" spans="5:7" x14ac:dyDescent="0.25">
@@ -503,10 +502,10 @@
         <v>2</v>
       </c>
       <c r="F35" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G35" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36" spans="5:7" x14ac:dyDescent="0.25">
@@ -514,10 +513,10 @@
         <v>3</v>
       </c>
       <c r="F36" t="s">
+        <v>7</v>
+      </c>
+      <c r="G36" t="s">
         <v>9</v>
-      </c>
-      <c r="G36" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>